<commit_message>
Update school presentations and add new files
</commit_message>
<xml_diff>
--- a/schools-presentations/A Semester - Programmatismos.xlsx
+++ b/schools-presentations/A Semester - Programmatismos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://moecyprus-my.sharepoint.com/personal/aaresti3_te_schools_ac_cy/Documents/Documents/education/schools-presentations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1717" documentId="11_F25DC773A252ABDACC10485521D851725BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36E5D0C3-8C58-49B8-8BCD-7019D9A3CB26}"/>
+  <xr:revisionPtr revIDLastSave="1718" documentId="11_F25DC773A252ABDACC10485521D851725BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C299AF1-F0B2-49E4-98A0-CFD7BCA66B9A}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="15" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="67080" yWindow="15" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="1" r:id="rId1"/>
@@ -1338,7 +1338,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1826" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1827" uniqueCount="380">
   <si>
     <t>Α Τάξη</t>
   </si>
@@ -2800,11 +2800,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2812,8 +2809,11 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3650,58 +3650,58 @@
   <sheetData>
     <row r="1" spans="1:60" s="3" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A1" s="28"/>
-      <c r="B1" s="43" t="s">
+      <c r="B1" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="44"/>
-      <c r="D1" s="43" t="s">
+      <c r="C1" s="43"/>
+      <c r="D1" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="43" t="s">
+      <c r="E1" s="43"/>
+      <c r="F1" s="42" t="s">
         <v>235</v>
       </c>
-      <c r="G1" s="44"/>
-      <c r="H1" s="43" t="s">
+      <c r="G1" s="43"/>
+      <c r="H1" s="42" t="s">
         <v>241</v>
       </c>
-      <c r="I1" s="44"/>
-      <c r="J1" s="43" t="s">
+      <c r="I1" s="43"/>
+      <c r="J1" s="42" t="s">
         <v>245</v>
       </c>
-      <c r="K1" s="44"/>
-      <c r="L1" s="43" t="s">
+      <c r="K1" s="43"/>
+      <c r="L1" s="42" t="s">
         <v>248</v>
       </c>
-      <c r="M1" s="44"/>
-      <c r="N1" s="43" t="s">
+      <c r="M1" s="43"/>
+      <c r="N1" s="42" t="s">
         <v>347</v>
       </c>
-      <c r="O1" s="44"/>
-      <c r="P1" s="43" t="s">
+      <c r="O1" s="43"/>
+      <c r="P1" s="42" t="s">
         <v>348</v>
       </c>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="43" t="s">
+      <c r="Q1" s="43"/>
+      <c r="R1" s="42" t="s">
         <v>350</v>
       </c>
-      <c r="S1" s="44"/>
-      <c r="T1" s="43" t="s">
+      <c r="S1" s="43"/>
+      <c r="T1" s="42" t="s">
         <v>351</v>
       </c>
-      <c r="U1" s="44"/>
-      <c r="V1" s="43" t="s">
+      <c r="U1" s="43"/>
+      <c r="V1" s="42" t="s">
         <v>352</v>
       </c>
-      <c r="W1" s="44"/>
-      <c r="X1" s="43" t="s">
+      <c r="W1" s="43"/>
+      <c r="X1" s="42" t="s">
         <v>353</v>
       </c>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="43" t="s">
+      <c r="Y1" s="43"/>
+      <c r="Z1" s="42" t="s">
         <v>354</v>
       </c>
-      <c r="AA1" s="44"/>
+      <c r="AA1" s="43"/>
       <c r="AB1" s="29"/>
       <c r="AC1" s="29"/>
       <c r="AD1" s="29"/>
@@ -3954,7 +3954,7 @@
       <c r="N6" s="23" t="s">
         <v>379</v>
       </c>
-      <c r="O6" s="45" t="s">
+      <c r="O6" s="41" t="s">
         <v>374</v>
       </c>
       <c r="P6" s="25" t="s">
@@ -4022,7 +4022,7 @@
       <c r="N7" s="23" t="s">
         <v>345</v>
       </c>
-      <c r="O7" s="45" t="s">
+      <c r="O7" s="41" t="s">
         <v>374</v>
       </c>
       <c r="X7" s="39" t="s">
@@ -4139,7 +4139,7 @@
       <c r="N12" s="23" t="s">
         <v>294</v>
       </c>
-      <c r="O12" s="45" t="s">
+      <c r="O12" s="41" t="s">
         <v>369</v>
       </c>
       <c r="V12" s="39" t="s">
@@ -4501,11 +4501,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="V1:W1"/>
-    <mergeCell ref="X1:Y1"/>
-    <mergeCell ref="Z1:AA1"/>
     <mergeCell ref="P1:Q1"/>
     <mergeCell ref="L1:M1"/>
     <mergeCell ref="N1:O1"/>
@@ -4514,6 +4509,11 @@
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="Z1:AA1"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4560,26 +4560,26 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="F2" s="41" t="s">
+      <c r="F2" s="44" t="s">
         <v>285</v>
       </c>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41" t="s">
+      <c r="G2" s="44"/>
+      <c r="H2" s="44" t="s">
         <v>286</v>
       </c>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41" t="s">
+      <c r="I2" s="44"/>
+      <c r="J2" s="44" t="s">
         <v>296</v>
       </c>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41" t="s">
+      <c r="K2" s="44"/>
+      <c r="L2" s="44" t="s">
         <v>322</v>
       </c>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41" t="s">
+      <c r="M2" s="44"/>
+      <c r="N2" s="44" t="s">
         <v>367</v>
       </c>
-      <c r="O2" s="41"/>
+      <c r="O2" s="44"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
@@ -6012,26 +6012,26 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="F2" s="41" t="s">
+      <c r="F2" s="44" t="s">
         <v>285</v>
       </c>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41" t="s">
+      <c r="G2" s="44"/>
+      <c r="H2" s="44" t="s">
         <v>286</v>
       </c>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41" t="s">
+      <c r="I2" s="44"/>
+      <c r="J2" s="44" t="s">
         <v>298</v>
       </c>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41" t="s">
+      <c r="K2" s="44"/>
+      <c r="L2" s="44" t="s">
         <v>322</v>
       </c>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41" t="s">
+      <c r="M2" s="44"/>
+      <c r="N2" s="44" t="s">
         <v>367</v>
       </c>
-      <c r="O2" s="41"/>
+      <c r="O2" s="44"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
@@ -7075,26 +7075,26 @@
       <c r="D1" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="41" t="s">
+      <c r="G1" s="44" t="s">
         <v>285</v>
       </c>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41" t="s">
+      <c r="H1" s="44"/>
+      <c r="I1" s="44" t="s">
         <v>286</v>
       </c>
-      <c r="J1" s="41"/>
-      <c r="K1" s="41" t="s">
+      <c r="J1" s="44"/>
+      <c r="K1" s="44" t="s">
         <v>298</v>
       </c>
-      <c r="L1" s="41"/>
-      <c r="M1" s="42" t="s">
+      <c r="L1" s="44"/>
+      <c r="M1" s="45" t="s">
         <v>328</v>
       </c>
-      <c r="N1" s="42"/>
-      <c r="O1" s="41" t="s">
+      <c r="N1" s="45"/>
+      <c r="O1" s="44" t="s">
         <v>367</v>
       </c>
-      <c r="P1" s="41"/>
+      <c r="P1" s="44"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
@@ -8824,18 +8824,18 @@
       <c r="D1" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="41" t="s">
+      <c r="E1" s="44" t="s">
         <v>285</v>
       </c>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41" t="s">
+      <c r="F1" s="44"/>
+      <c r="G1" s="44" t="s">
         <v>286</v>
       </c>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41" t="s">
+      <c r="H1" s="44"/>
+      <c r="I1" s="44" t="s">
         <v>298</v>
       </c>
-      <c r="J1" s="41"/>
+      <c r="J1" s="44"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4">
@@ -9671,7 +9671,9 @@
       <c r="D51" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="E51" s="20"/>
+      <c r="E51" s="6" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="4">

</xml_diff>

<commit_message>
lots of new staff
</commit_message>
<xml_diff>
--- a/schools-presentations/A Semester - Programmatismos.xlsx
+++ b/schools-presentations/A Semester - Programmatismos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://moecyprus-my.sharepoint.com/personal/aaresti3_te_schools_ac_cy/Documents/Documents/education/schools-presentations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1861" documentId="11_F25DC773A252ABDACC10485521D851725BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB0BECB4-FB79-4097-8189-605DC9F4E3FE}"/>
+  <xr:revisionPtr revIDLastSave="1880" documentId="11_F25DC773A252ABDACC10485521D851725BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61A2874D-444F-480B-9C1A-7110F256F582}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="15" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="67080" yWindow="15" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="1" r:id="rId1"/>
@@ -1311,7 +1311,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1866" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1870" uniqueCount="394">
   <si>
     <t>Α Τάξη</t>
   </si>
@@ -2538,6 +2538,21 @@
   </si>
   <si>
     <t>B41M14 - Επεξεργασία Γραφημάτων</t>
+  </si>
+  <si>
+    <t>ΣΧΟΛΙΚΗ ΓΙΟΡΤΗ</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>26-30/10 2026</t>
+  </si>
+  <si>
+    <t>hw ask.7-13, p146, via email</t>
+  </si>
+  <si>
+    <t>hw. Ex 1-17, A52M3</t>
   </si>
 </sst>
 </file>
@@ -2771,7 +2786,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2908,6 +2923,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2919,6 +2937,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3746,58 +3767,58 @@
   <sheetData>
     <row r="1" spans="1:60" s="3" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A1" s="28"/>
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="51"/>
-      <c r="D1" s="50" t="s">
+      <c r="C1" s="52"/>
+      <c r="D1" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="51"/>
-      <c r="F1" s="50" t="s">
+      <c r="E1" s="52"/>
+      <c r="F1" s="51" t="s">
         <v>233</v>
       </c>
-      <c r="G1" s="51"/>
-      <c r="H1" s="50" t="s">
+      <c r="G1" s="52"/>
+      <c r="H1" s="51" t="s">
         <v>239</v>
       </c>
-      <c r="I1" s="51"/>
-      <c r="J1" s="50" t="s">
+      <c r="I1" s="52"/>
+      <c r="J1" s="51" t="s">
         <v>243</v>
       </c>
-      <c r="K1" s="51"/>
-      <c r="L1" s="50" t="s">
+      <c r="K1" s="52"/>
+      <c r="L1" s="51" t="s">
         <v>246</v>
       </c>
-      <c r="M1" s="51"/>
-      <c r="N1" s="50" t="s">
+      <c r="M1" s="52"/>
+      <c r="N1" s="51" t="s">
         <v>345</v>
       </c>
-      <c r="O1" s="51"/>
-      <c r="P1" s="50" t="s">
+      <c r="O1" s="52"/>
+      <c r="P1" s="51" t="s">
         <v>346</v>
       </c>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="50" t="s">
+      <c r="Q1" s="52"/>
+      <c r="R1" s="51" t="s">
         <v>348</v>
       </c>
-      <c r="S1" s="51"/>
-      <c r="T1" s="50" t="s">
+      <c r="S1" s="52"/>
+      <c r="T1" s="51" t="s">
         <v>349</v>
       </c>
-      <c r="U1" s="51"/>
-      <c r="V1" s="50" t="s">
+      <c r="U1" s="52"/>
+      <c r="V1" s="51" t="s">
         <v>350</v>
       </c>
-      <c r="W1" s="51"/>
-      <c r="X1" s="50" t="s">
+      <c r="W1" s="52"/>
+      <c r="X1" s="51" t="s">
         <v>351</v>
       </c>
-      <c r="Y1" s="51"/>
-      <c r="Z1" s="50" t="s">
+      <c r="Y1" s="52"/>
+      <c r="Z1" s="51" t="s">
         <v>352</v>
       </c>
-      <c r="AA1" s="51"/>
+      <c r="AA1" s="52"/>
       <c r="AB1" s="29"/>
       <c r="AC1" s="29"/>
       <c r="AD1" s="29"/>
@@ -4012,7 +4033,7 @@
       <c r="O5" s="23" t="s">
         <v>371</v>
       </c>
-      <c r="P5" s="25" t="s">
+      <c r="P5" s="23" t="s">
         <v>353</v>
       </c>
       <c r="Q5" s="44" t="s">
@@ -4219,7 +4240,7 @@
       <c r="P11" s="23" t="s">
         <v>323</v>
       </c>
-      <c r="Q11" s="45" t="s">
+      <c r="Q11" s="50" t="s">
         <v>282</v>
       </c>
       <c r="R11" s="25" t="s">
@@ -4352,8 +4373,8 @@
       <c r="P13" s="23" t="s">
         <v>323</v>
       </c>
-      <c r="Q13" s="25" t="s">
-        <v>378</v>
+      <c r="Q13" s="23" t="s">
+        <v>390</v>
       </c>
       <c r="R13" s="25" t="s">
         <v>388</v>
@@ -4379,12 +4400,12 @@
         <v>236</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.5">
       <c r="H17" s="33" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="28.7" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:20" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A18" s="30" t="s">
         <v>14</v>
       </c>
@@ -4430,7 +4451,7 @@
       <c r="O18" s="23" t="s">
         <v>372</v>
       </c>
-      <c r="P18" s="36" t="s">
+      <c r="P18" s="23" t="s">
         <v>247</v>
       </c>
       <c r="Q18" s="27" t="s">
@@ -4440,7 +4461,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="28.7" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:20" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A19" s="30" t="s">
         <v>16</v>
       </c>
@@ -4486,17 +4507,20 @@
       <c r="O19" s="23" t="s">
         <v>372</v>
       </c>
-      <c r="P19" s="36" t="s">
-        <v>247</v>
+      <c r="P19" s="50" t="s">
+        <v>389</v>
       </c>
       <c r="Q19" s="27" t="s">
         <v>244</v>
       </c>
-      <c r="R19" s="27" t="s">
+      <c r="R19" s="36" t="s">
+        <v>247</v>
+      </c>
+      <c r="S19" s="27" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="28.7" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:20" ht="28.7" x14ac:dyDescent="0.5">
       <c r="A20" s="30" t="s">
         <v>15</v>
       </c>
@@ -4542,20 +4566,23 @@
       <c r="O20" s="23" t="s">
         <v>242</v>
       </c>
-      <c r="P20" s="36" t="s">
+      <c r="P20" s="50" t="s">
+        <v>389</v>
+      </c>
+      <c r="Q20" s="36" t="s">
         <v>295</v>
       </c>
-      <c r="Q20" s="36" t="s">
+      <c r="R20" s="36" t="s">
         <v>247</v>
       </c>
-      <c r="R20" s="27" t="s">
+      <c r="S20" s="27" t="s">
         <v>244</v>
       </c>
-      <c r="S20" s="27" t="s">
+      <c r="T20" s="27" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.5">
       <c r="B21" s="32"/>
       <c r="C21" s="34"/>
       <c r="D21" s="35"/>
@@ -4565,7 +4592,7 @@
       <c r="H21" s="23"/>
       <c r="I21" s="26"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.5">
       <c r="A22" s="30" t="s">
         <v>10</v>
       </c>
@@ -4601,27 +4628,27 @@
         <v>374</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.5">
       <c r="B23" s="32"/>
       <c r="C23" s="32"/>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.5">
       <c r="B24" s="32"/>
       <c r="C24" s="32"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.5">
       <c r="B25" s="37"/>
       <c r="C25" s="25" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.5">
       <c r="B26" s="34"/>
       <c r="C26" s="25" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.5">
       <c r="B27" s="27"/>
       <c r="C27" s="25" t="s">
         <v>29</v>
@@ -4629,19 +4656,19 @@
       <c r="P27" s="43"/>
       <c r="Q27" s="43"/>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.5">
       <c r="O28" s="41"/>
       <c r="R28" s="42"/>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.5">
       <c r="O29" s="41"/>
       <c r="R29" s="42"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.5">
       <c r="O30" s="41"/>
       <c r="R30" s="42"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.5">
       <c r="B31" s="25" t="s">
         <v>21</v>
       </c>
@@ -4654,7 +4681,7 @@
       <c r="O31" s="41"/>
       <c r="R31" s="42"/>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.5">
       <c r="B32" s="25" t="s">
         <v>22</v>
       </c>
@@ -4737,7 +4764,7 @@
     <col min="11" max="11" width="18.9375" style="4" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.64453125" style="4" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="16.87890625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.05859375" style="4"/>
+    <col min="14" max="14" width="17.64453125" style="4" customWidth="1"/>
     <col min="15" max="15" width="16.87890625" style="4" customWidth="1"/>
     <col min="16" max="16384" width="9.05859375" style="4"/>
   </cols>
@@ -4757,26 +4784,26 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="53" t="s">
         <v>283</v>
       </c>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52" t="s">
+      <c r="G2" s="53"/>
+      <c r="H2" s="53" t="s">
         <v>284</v>
       </c>
-      <c r="I2" s="52"/>
-      <c r="J2" s="52" t="s">
+      <c r="I2" s="53"/>
+      <c r="J2" s="53" t="s">
         <v>294</v>
       </c>
-      <c r="K2" s="52"/>
-      <c r="L2" s="52" t="s">
+      <c r="K2" s="53"/>
+      <c r="L2" s="53" t="s">
         <v>320</v>
       </c>
-      <c r="M2" s="52"/>
-      <c r="N2" s="52" t="s">
-        <v>365</v>
-      </c>
-      <c r="O2" s="52"/>
+      <c r="M2" s="53"/>
+      <c r="N2" s="53" t="s">
+        <v>391</v>
+      </c>
+      <c r="O2" s="53"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
@@ -5103,7 +5130,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:15" ht="31.35" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="4" t="s">
         <v>72</v>
       </c>
@@ -5121,6 +5148,9 @@
       </c>
       <c r="L15" s="4" t="s">
         <v>328</v>
+      </c>
+      <c r="N15" s="55" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.55000000000000004">
@@ -6177,26 +6207,26 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="53" t="s">
         <v>283</v>
       </c>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52" t="s">
+      <c r="G2" s="53"/>
+      <c r="H2" s="53" t="s">
         <v>284</v>
       </c>
-      <c r="I2" s="52"/>
-      <c r="J2" s="52" t="s">
+      <c r="I2" s="53"/>
+      <c r="J2" s="53" t="s">
         <v>296</v>
       </c>
-      <c r="K2" s="52"/>
-      <c r="L2" s="52" t="s">
+      <c r="K2" s="53"/>
+      <c r="L2" s="53" t="s">
         <v>320</v>
       </c>
-      <c r="M2" s="52"/>
-      <c r="N2" s="52" t="s">
+      <c r="M2" s="53"/>
+      <c r="N2" s="53" t="s">
         <v>365</v>
       </c>
-      <c r="O2" s="52"/>
+      <c r="O2" s="53"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
@@ -7240,26 +7270,26 @@
       <c r="D1" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="52" t="s">
+      <c r="G1" s="53" t="s">
         <v>283</v>
       </c>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52" t="s">
+      <c r="H1" s="53"/>
+      <c r="I1" s="53" t="s">
         <v>284</v>
       </c>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52" t="s">
+      <c r="J1" s="53"/>
+      <c r="K1" s="53" t="s">
         <v>296</v>
       </c>
-      <c r="L1" s="52"/>
-      <c r="M1" s="53" t="s">
+      <c r="L1" s="53"/>
+      <c r="M1" s="54" t="s">
         <v>326</v>
       </c>
-      <c r="N1" s="53"/>
-      <c r="O1" s="52" t="s">
+      <c r="N1" s="54"/>
+      <c r="O1" s="53" t="s">
         <v>365</v>
       </c>
-      <c r="P1" s="52"/>
+      <c r="P1" s="53"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
@@ -9086,18 +9116,18 @@
       <c r="D1" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="52" t="s">
+      <c r="E1" s="53" t="s">
         <v>283</v>
       </c>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52" t="s">
+      <c r="F1" s="53"/>
+      <c r="G1" s="53" t="s">
         <v>284</v>
       </c>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52" t="s">
+      <c r="H1" s="53"/>
+      <c r="I1" s="53" t="s">
         <v>296</v>
       </c>
-      <c r="J1" s="52"/>
+      <c r="J1" s="53"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4">
@@ -9211,7 +9241,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FEE7927-B2CB-4F8C-B929-249864A39417}">
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr defaultColWidth="9.05859375" defaultRowHeight="15.7" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="8.3515625" style="4" bestFit="1" customWidth="1"/>
@@ -9220,10 +9250,11 @@
     <col min="4" max="4" width="14.17578125" style="4" customWidth="1"/>
     <col min="5" max="5" width="10.234375" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.41015625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.05859375" style="4"/>
+    <col min="7" max="7" width="14.87890625" style="4" customWidth="1"/>
+    <col min="8" max="16384" width="9.05859375" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="7" t="s">
         <v>57</v>
       </c>
@@ -9237,7 +9268,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
         <v>121</v>
       </c>
@@ -9248,7 +9279,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="4">
         <v>9285104</v>
       </c>
@@ -9265,7 +9296,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="4">
         <v>8324104</v>
       </c>
@@ -9282,7 +9313,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="4">
         <v>6811804</v>
       </c>
@@ -9297,7 +9328,7 @@
       </c>
       <c r="E6" s="20"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="4">
         <v>5436904</v>
       </c>
@@ -9314,7 +9345,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="4">
         <v>7025704</v>
       </c>
@@ -9331,7 +9362,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="4">
         <v>8435804</v>
       </c>
@@ -9348,7 +9379,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="4">
         <v>5069104</v>
       </c>
@@ -9365,7 +9396,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="4">
         <v>5222304</v>
       </c>
@@ -9382,7 +9413,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="4">
         <v>1981204</v>
       </c>
@@ -9399,7 +9430,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="4">
         <v>3766704</v>
       </c>
@@ -9416,12 +9447,15 @@
         <v>171</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:7" ht="47" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="4" t="s">
         <v>72</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>276</v>
+      </c>
+      <c r="G16" s="55" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -10856,7 +10890,7 @@
         <v>15</v>
       </c>
       <c r="E20" t="s">
-        <v>309</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.5">

</xml_diff>